<commit_message>
Regelboken följer trycket; BTA-tabell, BYA-gräns och 'bruttototalarea' bekräftade
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/PU_BTA.xlsx
+++ b/kortdata/PU_BTA.xlsx
@@ -1242,7 +1242,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1377,17 +1377,29 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Tabellrubriken är tryckt 'bruttototalarea' (vanligen 'bruttoarea').</t>
+          <t>Tabellrubriken 'bruttototalarea' är avsiktlig (bekräftat av användaren).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Klasstabell bekräftad</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Mot fysiskt kort: A 500-5000, B 5001-7000, C 7001-9000, D &gt;9000 kvm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Byggd med</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>verktyg/bygg_pu_bta_bya_excel.py</t>
         </is>

</xml_diff>